<commit_message>
Correción de orden de magnitud en el conjunto de datos que registra intereses por sobregiros
</commit_message>
<xml_diff>
--- a/docs/reportes/METRICAS_DESEMPENO.xlsx
+++ b/docs/reportes/METRICAS_DESEMPENO.xlsx
@@ -471,19 +471,19 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>06:02:47</t>
+          <t>06:37:12</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>06:02:47</t>
+          <t>06:37:12</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>0.2808</v>
+        <v>0.1693</v>
       </c>
       <c r="G2" t="n">
-        <v>4.25</v>
+        <v>3.81</v>
       </c>
     </row>
     <row r="3">
@@ -504,19 +504,19 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>06:02:47</t>
+          <t>06:37:12</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>06:02:49</t>
+          <t>06:37:14</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>1.9025</v>
+        <v>1.2118</v>
       </c>
       <c r="G3" t="n">
-        <v>28.77</v>
+        <v>27.29</v>
       </c>
     </row>
     <row r="4">
@@ -537,19 +537,19 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>06:02:49</t>
+          <t>06:37:14</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>06:02:49</t>
+          <t>06:37:14</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>0.0037</v>
+        <v>0.0021</v>
       </c>
       <c r="G4" t="n">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="5">
@@ -570,16 +570,16 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>06:02:49</t>
+          <t>06:37:14</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>06:02:49</t>
+          <t>06:37:14</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>0.0172</v>
+        <v>0.0117</v>
       </c>
       <c r="G5" t="n">
         <v>0.26</v>
@@ -603,19 +603,19 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>06:02:49</t>
+          <t>06:37:14</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>06:02:49</t>
+          <t>06:37:14</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>0.0183</v>
+        <v>0.0104</v>
       </c>
       <c r="G6" t="n">
-        <v>0.28</v>
+        <v>0.23</v>
       </c>
     </row>
     <row r="7">
@@ -636,19 +636,19 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>06:02:49</t>
+          <t>06:37:14</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>06:02:49</t>
+          <t>06:37:14</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>0.0142</v>
+        <v>0.0076</v>
       </c>
       <c r="G7" t="n">
-        <v>0.21</v>
+        <v>0.17</v>
       </c>
     </row>
     <row r="8">
@@ -669,19 +669,19 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>06:02:49</t>
+          <t>06:37:14</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>06:02:49</t>
+          <t>06:37:14</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>0.0987</v>
+        <v>0.0675</v>
       </c>
       <c r="G8" t="n">
-        <v>1.49</v>
+        <v>1.52</v>
       </c>
     </row>
     <row r="9">
@@ -702,19 +702,19 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>06:02:49</t>
+          <t>06:37:14</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>06:02:49</t>
+          <t>06:37:14</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>0.007</v>
+        <v>0.0067</v>
       </c>
       <c r="G9" t="n">
-        <v>0.11</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="10">
@@ -735,19 +735,19 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>06:02:49</t>
+          <t>06:37:14</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>06:02:50</t>
+          <t>06:37:14</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>0.7684</v>
+        <v>0.4107</v>
       </c>
       <c r="G10" t="n">
-        <v>11.62</v>
+        <v>9.25</v>
       </c>
     </row>
     <row r="11">
@@ -768,19 +768,19 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>06:02:50</t>
+          <t>06:37:14</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>06:02:50</t>
+          <t>06:37:15</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>0.4503</v>
+        <v>0.3058</v>
       </c>
       <c r="G11" t="n">
-        <v>6.81</v>
+        <v>6.89</v>
       </c>
     </row>
     <row r="12">
@@ -801,19 +801,19 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>06:02:50</t>
+          <t>06:37:15</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>06:02:51</t>
+          <t>06:37:15</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>0.2595</v>
+        <v>0.1484</v>
       </c>
       <c r="G12" t="n">
-        <v>3.92</v>
+        <v>3.34</v>
       </c>
     </row>
     <row r="13">
@@ -834,19 +834,19 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>06:02:51</t>
+          <t>06:37:15</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>06:02:51</t>
+          <t>06:37:15</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>0.3811</v>
+        <v>0.2408</v>
       </c>
       <c r="G13" t="n">
-        <v>5.76</v>
+        <v>5.42</v>
       </c>
     </row>
     <row r="14">
@@ -867,19 +867,19 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>06:02:51</t>
+          <t>06:37:15</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>06:02:51</t>
+          <t>06:37:15</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>0.3098</v>
+        <v>0.1895</v>
       </c>
       <c r="G14" t="n">
-        <v>4.68</v>
+        <v>4.27</v>
       </c>
     </row>
     <row r="15">
@@ -900,19 +900,19 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>06:02:51</t>
+          <t>06:37:15</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>06:02:52</t>
+          <t>06:37:15</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>0.2737</v>
+        <v>0.2111</v>
       </c>
       <c r="G15" t="n">
-        <v>4.14</v>
+        <v>4.75</v>
       </c>
     </row>
     <row r="16">
@@ -933,19 +933,19 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>06:02:52</t>
+          <t>06:37:15</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>06:02:52</t>
+          <t>06:37:16</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>0.3265</v>
+        <v>0.2576</v>
       </c>
       <c r="G16" t="n">
-        <v>4.94</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="17">
@@ -966,19 +966,19 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>06:02:52</t>
+          <t>06:37:16</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>06:02:52</t>
+          <t>06:37:16</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>0.4209</v>
+        <v>0.2852</v>
       </c>
       <c r="G17" t="n">
-        <v>6.36</v>
+        <v>6.42</v>
       </c>
     </row>
     <row r="18">
@@ -999,19 +999,19 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>06:02:52</t>
+          <t>06:37:16</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>06:02:53</t>
+          <t>06:37:16</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>0.3234</v>
+        <v>0.2514</v>
       </c>
       <c r="G18" t="n">
-        <v>4.89</v>
+        <v>5.66</v>
       </c>
     </row>
     <row r="19">
@@ -1032,19 +1032,19 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>06:02:53</t>
+          <t>06:37:16</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>06:02:53</t>
+          <t>06:37:16</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>0.3062</v>
+        <v>0.2265</v>
       </c>
       <c r="G19" t="n">
-        <v>4.63</v>
+        <v>5.1</v>
       </c>
     </row>
     <row r="20">
@@ -1065,19 +1065,19 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>06:02:53</t>
+          <t>06:37:16</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>06:02:53</t>
+          <t>06:37:17</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>0.206</v>
+        <v>0.1958</v>
       </c>
       <c r="G20" t="n">
-        <v>3.11</v>
+        <v>4.41</v>
       </c>
     </row>
     <row r="21">
@@ -1098,19 +1098,19 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>06:02:53</t>
+          <t>06:37:17</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>06:02:53</t>
+          <t>06:37:17</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>0.2456</v>
+        <v>0.23</v>
       </c>
       <c r="G21" t="n">
-        <v>3.71</v>
+        <v>5.18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>